<commit_message>
feat(rules/batch): incorporate MBA consulting teams into Rule 29 and update batch 392-407 to 23 effect sizes
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/392_398_399_403_407.xlsx
+++ b/03_Coding_Sheets/392_398_399_403_407.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AX24"/>
+  <dimension ref="A1:AX28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -848,7 +848,7 @@
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "2. Outdegree in internal network" x Col: "1. Hierarchical level" = .26 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "2. Outdegree in internal network" x Col: "1. Hierarchical level" = .26 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -992,7 +992,7 @@
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "3. Boundary spanning ties" x Col: "1. Hierarchical level" = .32 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "3. Boundary spanning ties" x Col: "1. Hierarchical level" = .32 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -1136,7 +1136,7 @@
       </c>
       <c r="AX6" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "4. Outdegree in extended network" x Col: "1. Hierarchical level" = .35 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "4. Outdegree in extended network" x Col: "1. Hierarchical level" = .35 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1280,7 @@
       </c>
       <c r="AX7" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "5. Boundary spanning orientation" x Col: "1. Hierarchical level" = .15 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "5. Boundary spanning orientation" x Col: "1. Hierarchical level" = .15 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -1424,7 +1424,7 @@
       </c>
       <c r="AX8" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "2. Outdegree in internal network" = .35 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "2. Outdegree in internal network" = .35 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -1568,7 +1568,7 @@
       </c>
       <c r="AX9" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "3. Boundary spanning ties" = .34 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "3. Boundary spanning ties" = .34 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -1708,11 +1708,11 @@
         <v>0.91</v>
       </c>
       <c r="AW10" t="n">
-        <v>0.42</v>
+        <v>0.4</v>
       </c>
       <c r="AX10" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "4. Outdegree in extended network" = .42 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "4. Outdegree in extended network" = .40 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -1852,11 +1852,11 @@
         <v>0.91</v>
       </c>
       <c r="AW11" t="n">
-        <v>0.14</v>
+        <v>0.16</v>
       </c>
       <c r="AX11" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "5. Boundary spanning orientation" = .14 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "5. Boundary spanning orientation" = .16 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -2001,11 +2001,11 @@
         <v>999</v>
       </c>
       <c r="AW12" t="n">
-        <v>0.32</v>
+        <v>0.58</v>
       </c>
       <c r="AX12" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "2. Outdegree in internal network" = .32 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "2. Outdegree in internal network" = .58 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -2150,11 +2150,11 @@
         <v>999</v>
       </c>
       <c r="AW13" t="n">
-        <v>0.32</v>
+        <v>0.51</v>
       </c>
       <c r="AX13" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "3. Boundary spanning ties" = .32 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "3. Boundary spanning ties" = .51 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -2299,11 +2299,11 @@
         <v>999</v>
       </c>
       <c r="AW14" t="n">
-        <v>0.39</v>
+        <v>0.63</v>
       </c>
       <c r="AX14" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "4. Outdegree in extended network" = .39 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "4. Outdegree in extended network" = .63 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -2448,11 +2448,11 @@
         <v>999</v>
       </c>
       <c r="AW15" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="AX15" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "5. Boundary spanning orientation" = .15 | Listwise N = 108 | Table Footnote: "Correlations above .20 are significant at .05 level."</t>
+          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "5. Boundary spanning orientation" = .17 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
         </is>
       </c>
     </row>
@@ -2475,12 +2475,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>2 = Longitudinal design</t>
-        </is>
-      </c>
-      <c r="R16" t="inlineStr">
-        <is>
-          <t>Two waves separated by a 3-month gap (T1: supportive coaching &amp; self-efficacy; T2: boundary-spanning behavior &amp; job satisfaction)</t>
+          <t>1 = Cross-sectional design</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2497,21 +2492,21 @@
         <v>170</v>
       </c>
       <c r="W16" t="n">
-        <v>41.92</v>
+        <v>39</v>
       </c>
       <c r="X16" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="Y16" t="n">
-        <v>9.039999999999999</v>
+        <v>6</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>Engineering and manufacturing employees (nonmanagement team members)</t>
+          <t>Engineers / Engineering employees</t>
         </is>
       </c>
       <c r="AA16" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="AB16" t="n">
         <v>1</v>
@@ -2524,19 +2519,14 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE16" t="inlineStr">
-        <is>
-          <t>Thirteen items selected from Ancona and Caldwell (1992) assessing ambassadorial (5 items), scouting (4 items), and task coordination (4 items) behaviors rated on a 5-point scale (1 = a very small extent to 5 = a very great extent).</t>
-        </is>
-      </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>Ancona and Caldwell’s (1992)</t>
+          <t>Marrone et al., 2007</t>
         </is>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>Thirteen-item scale based on Ancona and Caldwell (1992) assessing ambassadorial, scouting, and task coordination behaviors averaged to form three indicator variables for overall boundary-spanning behavior.</t>
+          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
         </is>
       </c>
       <c r="AH16" t="n">
@@ -2555,12 +2545,12 @@
       </c>
       <c r="AM16" t="inlineStr">
         <is>
-          <t>age in years</t>
+          <t>demographic question</t>
         </is>
       </c>
       <c r="AN16" t="inlineStr">
         <is>
-          <t>Chronological age measured in years.</t>
+          <t>Participant age in years measured as a continuous demographic variable.</t>
         </is>
       </c>
       <c r="AO16" t="inlineStr">
@@ -2569,13 +2559,13 @@
         </is>
       </c>
       <c r="AP16" t="n">
-        <v>2.62</v>
+        <v>3.48</v>
       </c>
       <c r="AQ16" t="n">
-        <v>0.83</v>
+        <v>0.65</v>
       </c>
       <c r="AR16" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.88</v>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
@@ -2583,10 +2573,10 @@
         </is>
       </c>
       <c r="AT16" t="n">
-        <v>41.92</v>
+        <v>39</v>
       </c>
       <c r="AU16" t="n">
-        <v>11.11</v>
+        <v>12</v>
       </c>
       <c r="AV16" t="n">
         <v>999</v>
@@ -2619,12 +2609,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>2 = Longitudinal design</t>
-        </is>
-      </c>
-      <c r="R17" t="inlineStr">
-        <is>
-          <t>Two waves separated by a 3-month gap (T1: supportive coaching &amp; self-efficacy; T2: boundary-spanning behavior &amp; job satisfaction)</t>
+          <t>1 = Cross-sectional design</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2641,21 +2626,21 @@
         <v>170</v>
       </c>
       <c r="W17" t="n">
-        <v>41.92</v>
+        <v>39</v>
       </c>
       <c r="X17" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="Y17" t="n">
-        <v>9.039999999999999</v>
+        <v>6</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>Engineering and manufacturing employees (nonmanagement team members)</t>
+          <t>Engineers / Engineering employees</t>
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="AB17" t="n">
         <v>1</v>
@@ -2668,19 +2653,14 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE17" t="inlineStr">
-        <is>
-          <t>Thirteen items selected from Ancona and Caldwell (1992) assessing ambassadorial (5 items), scouting (4 items), and task coordination (4 items) behaviors rated on a 5-point scale (1 = a very small extent to 5 = a very great extent).</t>
-        </is>
-      </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>Ancona and Caldwell’s (1992)</t>
+          <t>Marrone et al., 2007</t>
         </is>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>Thirteen-item scale based on Ancona and Caldwell (1992) assessing ambassadorial, scouting, and task coordination behaviors averaged to form three indicator variables for overall boundary-spanning behavior.</t>
+          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
         </is>
       </c>
       <c r="AH17" t="n">
@@ -2699,12 +2679,12 @@
       </c>
       <c r="AM17" t="inlineStr">
         <is>
-          <t>gender using male = 1 and female = 2</t>
+          <t>demographic question</t>
         </is>
       </c>
       <c r="AN17" t="inlineStr">
         <is>
-          <t>Dichotomous gender coded using male = 1 and female = 2.</t>
+          <t>Participant gender coded as female = 1 and male = 2.</t>
         </is>
       </c>
       <c r="AO17" t="inlineStr">
@@ -2713,13 +2693,13 @@
         </is>
       </c>
       <c r="AP17" t="n">
-        <v>2.62</v>
+        <v>3.48</v>
       </c>
       <c r="AQ17" t="n">
-        <v>0.83</v>
+        <v>0.65</v>
       </c>
       <c r="AR17" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.88</v>
       </c>
       <c r="AS17" t="inlineStr">
         <is>
@@ -2727,10 +2707,10 @@
         </is>
       </c>
       <c r="AT17" t="n">
-        <v>1.1</v>
+        <v>1.79</v>
       </c>
       <c r="AU17" t="n">
-        <v>0.3</v>
+        <v>0.41</v>
       </c>
       <c r="AV17" t="n">
         <v>999</v>
@@ -2763,12 +2743,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>2 = Longitudinal design</t>
-        </is>
-      </c>
-      <c r="R18" t="inlineStr">
-        <is>
-          <t>Two waves separated by a 3-month gap (T1: supportive coaching &amp; self-efficacy; T2: boundary-spanning behavior &amp; job satisfaction)</t>
+          <t>1 = Cross-sectional design</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2785,21 +2760,21 @@
         <v>170</v>
       </c>
       <c r="W18" t="n">
-        <v>41.92</v>
+        <v>39</v>
       </c>
       <c r="X18" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="Y18" t="n">
-        <v>9.039999999999999</v>
+        <v>6</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>Engineering and manufacturing employees (nonmanagement team members)</t>
+          <t>Engineers / Engineering employees</t>
         </is>
       </c>
       <c r="AA18" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="AB18" t="n">
         <v>1</v>
@@ -2812,19 +2787,14 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE18" t="inlineStr">
-        <is>
-          <t>Thirteen items selected from Ancona and Caldwell (1992) assessing ambassadorial (5 items), scouting (4 items), and task coordination (4 items) behaviors rated on a 5-point scale (1 = a very small extent to 5 = a very great extent).</t>
-        </is>
-      </c>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>Ancona and Caldwell’s (1992)</t>
+          <t>Marrone et al., 2007</t>
         </is>
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>Thirteen-item scale based on Ancona and Caldwell (1992) assessing ambassadorial, scouting, and task coordination behaviors averaged to form three indicator variables for overall boundary-spanning behavior.</t>
+          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
         </is>
       </c>
       <c r="AH18" t="n">
@@ -2843,7 +2813,7 @@
       </c>
       <c r="AM18" t="inlineStr">
         <is>
-          <t>ethnicity/race</t>
+          <t>demographic question</t>
         </is>
       </c>
       <c r="AN18" t="inlineStr">
@@ -2857,13 +2827,13 @@
         </is>
       </c>
       <c r="AP18" t="n">
-        <v>2.62</v>
+        <v>3.48</v>
       </c>
       <c r="AQ18" t="n">
-        <v>0.83</v>
+        <v>0.65</v>
       </c>
       <c r="AR18" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.88</v>
       </c>
       <c r="AS18" t="inlineStr">
         <is>
@@ -2907,12 +2877,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>2 = Longitudinal design</t>
-        </is>
-      </c>
-      <c r="R19" t="inlineStr">
-        <is>
-          <t>Two waves separated by a 3-month gap (T1: supportive coaching &amp; self-efficacy; T2: boundary-spanning behavior &amp; job satisfaction)</t>
+          <t>1 = Cross-sectional design</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2929,21 +2894,21 @@
         <v>170</v>
       </c>
       <c r="W19" t="n">
-        <v>41.92</v>
+        <v>39</v>
       </c>
       <c r="X19" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="Y19" t="n">
-        <v>9.039999999999999</v>
+        <v>6</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>Engineering and manufacturing employees (nonmanagement team members)</t>
+          <t>Engineers / Engineering employees</t>
         </is>
       </c>
       <c r="AA19" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="AB19" t="n">
         <v>1</v>
@@ -2956,19 +2921,14 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE19" t="inlineStr">
-        <is>
-          <t>Thirteen items selected from Ancona and Caldwell (1992) assessing ambassadorial (5 items), scouting (4 items), and task coordination (4 items) behaviors rated on a 5-point scale (1 = a very small extent to 5 = a very great extent).</t>
-        </is>
-      </c>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>Ancona and Caldwell’s (1992)</t>
+          <t>Marrone et al., 2007</t>
         </is>
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>Thirteen-item scale based on Ancona and Caldwell (1992) assessing ambassadorial, scouting, and task coordination behaviors averaged to form three indicator variables for overall boundary-spanning behavior.</t>
+          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
         </is>
       </c>
       <c r="AH19" t="n">
@@ -3006,13 +2966,13 @@
         </is>
       </c>
       <c r="AP19" t="n">
-        <v>2.62</v>
+        <v>3.48</v>
       </c>
       <c r="AQ19" t="n">
-        <v>0.83</v>
+        <v>0.65</v>
       </c>
       <c r="AR19" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.88</v>
       </c>
       <c r="AS19" t="inlineStr">
         <is>
@@ -3056,12 +3016,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>2 = Longitudinal design</t>
-        </is>
-      </c>
-      <c r="R20" t="inlineStr">
-        <is>
-          <t>Two waves separated by a 3-month gap (T1: supportive coaching &amp; self-efficacy; T2: boundary-spanning behavior &amp; job satisfaction)</t>
+          <t>1 = Cross-sectional design</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -3078,21 +3033,21 @@
         <v>170</v>
       </c>
       <c r="W20" t="n">
-        <v>41.92</v>
+        <v>39</v>
       </c>
       <c r="X20" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="Y20" t="n">
-        <v>9.039999999999999</v>
+        <v>6</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>Engineering and manufacturing employees (nonmanagement team members)</t>
+          <t>Engineers / Engineering employees</t>
         </is>
       </c>
       <c r="AA20" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="AB20" t="n">
         <v>1</v>
@@ -3105,19 +3060,14 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE20" t="inlineStr">
-        <is>
-          <t>Thirteen items selected from Ancona and Caldwell (1992) assessing ambassadorial (5 items), scouting (4 items), and task coordination (4 items) behaviors rated on a 5-point scale (1 = a very small extent to 5 = a very great extent).</t>
-        </is>
-      </c>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>Ancona and Caldwell’s (1992)</t>
+          <t>Marrone et al., 2007</t>
         </is>
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>Thirteen-item scale based on Ancona and Caldwell (1992) assessing ambassadorial, scouting, and task coordination behaviors averaged to form three indicator variables for overall boundary-spanning behavior.</t>
+          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
         </is>
       </c>
       <c r="AH20" t="n">
@@ -3150,13 +3100,13 @@
         </is>
       </c>
       <c r="AP20" t="n">
-        <v>2.62</v>
+        <v>3.48</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0.83</v>
+        <v>0.65</v>
       </c>
       <c r="AR20" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.88</v>
       </c>
       <c r="AS20" t="inlineStr">
         <is>
@@ -3200,12 +3150,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>2 = Longitudinal design</t>
-        </is>
-      </c>
-      <c r="R21" t="inlineStr">
-        <is>
-          <t>Two waves separated by a 3-month gap (T1: supportive coaching &amp; self-efficacy; T2: boundary-spanning behavior &amp; job satisfaction)</t>
+          <t>1 = Cross-sectional design</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -3222,21 +3167,21 @@
         <v>170</v>
       </c>
       <c r="W21" t="n">
-        <v>41.92</v>
+        <v>39</v>
       </c>
       <c r="X21" t="n">
-        <v>10</v>
+        <v>21</v>
       </c>
       <c r="Y21" t="n">
-        <v>9.039999999999999</v>
+        <v>6</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>Engineering and manufacturing employees (nonmanagement team members)</t>
+          <t>Engineers / Engineering employees</t>
         </is>
       </c>
       <c r="AA21" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="AB21" t="n">
         <v>1</v>
@@ -3249,19 +3194,14 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AE21" t="inlineStr">
-        <is>
-          <t>Thirteen items selected from Ancona and Caldwell (1992) assessing ambassadorial (5 items), scouting (4 items), and task coordination (4 items) behaviors rated on a 5-point scale (1 = a very small extent to 5 = a very great extent).</t>
-        </is>
-      </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>Ancona and Caldwell’s (1992)</t>
+          <t>Marrone et al., 2007</t>
         </is>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>Thirteen-item scale based on Ancona and Caldwell (1992) assessing ambassadorial, scouting, and task coordination behaviors averaged to form three indicator variables for overall boundary-spanning behavior.</t>
+          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
         </is>
       </c>
       <c r="AH21" t="n">
@@ -3294,13 +3234,13 @@
         </is>
       </c>
       <c r="AP21" t="n">
-        <v>2.62</v>
+        <v>3.48</v>
       </c>
       <c r="AQ21" t="n">
-        <v>0.83</v>
+        <v>0.65</v>
       </c>
       <c r="AR21" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.88</v>
       </c>
       <c r="AS21" t="inlineStr">
         <is>
@@ -3334,19 +3274,138 @@
       <c r="B22" t="n">
         <v>399</v>
       </c>
+      <c r="D22" t="n">
+        <v>1</v>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0 = exclude</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>2 = Non-employee samples</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>The study evaluates a sample of 190 MBA students across 31 consulting teams participating in coursework consulting engagements as part of their academic degree requirements. Under BSMA Rule 29, student samples in academic coursework or classroom projects are non-worker populations strictly excluded under Code 2. Verbatim Evidence: [p. 1428] "We collected data from a sample of 190 MBA students, comprising 31 consulting teams [5-7 members per team), at a large mid-Atlantic university. The sample was a realistic and appropriate research setting for exploring boundary spanning as the teams were highly reliant on external sources for carrying out their work. Every second-year MBA student was required to participate in an intensive, semester-long, actual consulting engagement with a real organization. Participants were assigned to consulting teams on the basis of their concentration areas and domains of experience."</t>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S22" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="T22" t="inlineStr">
+        <is>
+          <t>Mid-Atlantic United States</t>
+        </is>
+      </c>
+      <c r="U22" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V22" t="n">
+        <v>190</v>
+      </c>
+      <c r="W22" t="n">
+        <v>999</v>
+      </c>
+      <c r="X22" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y22" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z22" t="inlineStr">
+        <is>
+          <t>MBA students (consulting teams)</t>
+        </is>
+      </c>
+      <c r="AA22" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC22" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD22" t="inlineStr">
+        <is>
+          <t>2 = Peer-report</t>
+        </is>
+      </c>
+      <c r="AE22" t="inlineStr">
+        <is>
+          <t>Peer ratings across consulting teammates justified by median rwg = 0.80, ICC(1) = 0.28, ICC(2) = 0.71.</t>
+        </is>
+      </c>
+      <c r="AF22" t="inlineStr">
+        <is>
+          <t>Ancona and Caldwell's (1992)</t>
+        </is>
+      </c>
+      <c r="AG22" t="inlineStr">
+        <is>
+          <t>Six items adapted from Ancona and Caldwell (1992) capturing individual team member boundary-spanning behaviors across client, faculty advisor, and external organizational interfaces.</t>
+        </is>
+      </c>
+      <c r="AH22" t="n">
+        <v>6</v>
+      </c>
+      <c r="AI22" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ22" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK22" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM22" t="inlineStr">
+        <is>
+          <t>role theory</t>
+        </is>
+      </c>
+      <c r="AN22" t="inlineStr">
+        <is>
+          <t>Six items assessing the extent to which participants perceived boundary-spanning behaviors as an expected part of their role responsibilities (alpha = 0.86).</t>
+        </is>
+      </c>
+      <c r="AO22" t="inlineStr">
+        <is>
+          <t>Boundary-spanning behavior</t>
+        </is>
+      </c>
+      <c r="AP22" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AQ22" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AR22" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AS22" t="inlineStr">
+        <is>
+          <t>Boundary-spanning role</t>
+        </is>
+      </c>
+      <c r="AT22" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="AU22" t="n">
+        <v>0.82</v>
+      </c>
+      <c r="AV22" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AW22" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AX22" t="inlineStr">
+        <is>
+          <t>Table 1 (p. 1432) | Row: "2. Boundary-spanning role" x Col: "1. Boundary-spanning behavior" = .40** | Pairwise n = 186 (Total N = 190) | Table Footnote: "* p &lt; .05 ** p &lt; .01"</t>
         </is>
       </c>
     </row>
@@ -3357,21 +3416,140 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>403</v>
+        <v>399</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0 = exclude</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr">
-        <is>
-          <t>3 = Non-individual level (team/firm/org analysis)</t>
-        </is>
-      </c>
-      <c r="P23" t="inlineStr">
-        <is>
-          <t>The unit of statistical analysis is the business organization (N = 62 publicly held U.S. corporations on the Russell 1000 index). The 62 Public Affairs Managers served merely as single key informants evaluating the firm's macro-level relationships with public interest groups using firm-referent items (e.g., The firm avoids close contact with this socio-political actor), violating Screening Rule 4 and Rule 5 (Proxy Guardrail). Verbatim Evidence: [p. 58] "A survey of 62 Public Affairs Managers in publicly held U.S. corporations finds that organizations adopt relational styles similar to those theorized in studies of inter-organizational conflict, organizational communication and stakeholder management." [p. 62] "The organizations participating in this study were large, U.S. companies listed on the Russell 1000 index from a variety of industries... A limitation of the study is that only one manager responded for each organization. The vulnerability inherent in this practice is that the manager's understanding reflected in the survey may not be representative of the organization's practices."</t>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S23" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>Mid-Atlantic United States</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V23" t="n">
+        <v>190</v>
+      </c>
+      <c r="W23" t="n">
+        <v>999</v>
+      </c>
+      <c r="X23" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y23" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>MBA students (consulting teams)</t>
+        </is>
+      </c>
+      <c r="AA23" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC23" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD23" t="inlineStr">
+        <is>
+          <t>2 = Peer-report</t>
+        </is>
+      </c>
+      <c r="AE23" t="inlineStr">
+        <is>
+          <t>Peer ratings across consulting teammates justified by median rwg = 0.80, ICC(1) = 0.28, ICC(2) = 0.71.</t>
+        </is>
+      </c>
+      <c r="AF23" t="inlineStr">
+        <is>
+          <t>Ancona and Caldwell's (1992)</t>
+        </is>
+      </c>
+      <c r="AG23" t="inlineStr">
+        <is>
+          <t>Six items adapted from Ancona and Caldwell (1992) capturing individual team member boundary-spanning behaviors across client, faculty advisor, and external organizational interfaces.</t>
+        </is>
+      </c>
+      <c r="AH23" t="n">
+        <v>8</v>
+      </c>
+      <c r="AI23" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ23" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK23" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM23" t="inlineStr">
+        <is>
+          <t>Parker's (1998)</t>
+        </is>
+      </c>
+      <c r="AN23" t="inlineStr">
+        <is>
+          <t>Eight-item scale adapted from Parker (1998) role breadth self-efficacy measuring confidence in engaging in boundary-spanning behaviors (alpha = 0.92).</t>
+        </is>
+      </c>
+      <c r="AO23" t="inlineStr">
+        <is>
+          <t>Boundary-spanning behavior</t>
+        </is>
+      </c>
+      <c r="AP23" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AQ23" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AR23" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AS23" t="inlineStr">
+        <is>
+          <t>Boundary-spanning self-efficacy</t>
+        </is>
+      </c>
+      <c r="AT23" t="n">
+        <v>4.07</v>
+      </c>
+      <c r="AU23" t="n">
+        <v>0.6899999999999999</v>
+      </c>
+      <c r="AV23" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="AW23" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="AX23" t="inlineStr">
+        <is>
+          <t>Table 1 (p. 1432) | Row: "3. Boundary-spanning self-efficacy" x Col: "1. Boundary-spanning behavior" = .25** | Pairwise n = 190 (Total N = 190) | Table Footnote: "* p &lt; .05 ** p &lt; .01"</t>
         </is>
       </c>
     </row>
@@ -3382,19 +3560,481 @@
         </is>
       </c>
       <c r="B24" t="n">
+        <v>399</v>
+      </c>
+      <c r="D24" t="n">
+        <v>3</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S24" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="T24" t="inlineStr">
+        <is>
+          <t>Mid-Atlantic United States</t>
+        </is>
+      </c>
+      <c r="U24" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V24" t="n">
+        <v>190</v>
+      </c>
+      <c r="W24" t="n">
+        <v>999</v>
+      </c>
+      <c r="X24" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y24" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z24" t="inlineStr">
+        <is>
+          <t>MBA students (consulting teams)</t>
+        </is>
+      </c>
+      <c r="AA24" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC24" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD24" t="inlineStr">
+        <is>
+          <t>2 = Peer-report</t>
+        </is>
+      </c>
+      <c r="AE24" t="inlineStr">
+        <is>
+          <t>Peer ratings across consulting teammates justified by median rwg = 0.80, ICC(1) = 0.28, ICC(2) = 0.71.</t>
+        </is>
+      </c>
+      <c r="AF24" t="inlineStr">
+        <is>
+          <t>Ancona and Caldwell's (1992)</t>
+        </is>
+      </c>
+      <c r="AG24" t="inlineStr">
+        <is>
+          <t>Six items adapted from Ancona and Caldwell (1992) capturing individual team member boundary-spanning behaviors across client, faculty advisor, and external organizational interfaces.</t>
+        </is>
+      </c>
+      <c r="AH24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI24" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ24" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK24" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM24" t="inlineStr">
+        <is>
+          <t>Williams &amp; O'Reilly (1998)</t>
+        </is>
+      </c>
+      <c r="AN24" t="inlineStr">
+        <is>
+          <t>Demographic control variable coded as Asian = 1 and other = 0.</t>
+        </is>
+      </c>
+      <c r="AO24" t="inlineStr">
+        <is>
+          <t>Boundary-spanning behavior</t>
+        </is>
+      </c>
+      <c r="AP24" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AQ24" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AR24" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AS24" t="inlineStr">
+        <is>
+          <t>Asian ethnicity</t>
+        </is>
+      </c>
+      <c r="AT24" t="n">
+        <v>0.31</v>
+      </c>
+      <c r="AU24" t="n">
+        <v>0.46</v>
+      </c>
+      <c r="AV24" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW24" t="n">
+        <v>-0.23</v>
+      </c>
+      <c r="AX24" t="inlineStr">
+        <is>
+          <t>Table 1 (p. 1432) | Row: "4. Asian ethnicity" x Col: "1. Boundary-spanning behavior" = -.23** | Pairwise n = 182 (Total N = 190) | Table Footnote: "* p &lt; .05 ** p &lt; .01"</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>399</v>
+      </c>
+      <c r="D25" t="n">
+        <v>4</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="T25" t="inlineStr">
+        <is>
+          <t>Mid-Atlantic United States</t>
+        </is>
+      </c>
+      <c r="U25" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V25" t="n">
+        <v>190</v>
+      </c>
+      <c r="W25" t="n">
+        <v>999</v>
+      </c>
+      <c r="X25" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y25" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z25" t="inlineStr">
+        <is>
+          <t>MBA students (consulting teams)</t>
+        </is>
+      </c>
+      <c r="AA25" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC25" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD25" t="inlineStr">
+        <is>
+          <t>2 = Peer-report</t>
+        </is>
+      </c>
+      <c r="AE25" t="inlineStr">
+        <is>
+          <t>Peer ratings across consulting teammates justified by median rwg = 0.80, ICC(1) = 0.28, ICC(2) = 0.71.</t>
+        </is>
+      </c>
+      <c r="AF25" t="inlineStr">
+        <is>
+          <t>Ancona and Caldwell's (1992)</t>
+        </is>
+      </c>
+      <c r="AG25" t="inlineStr">
+        <is>
+          <t>Six items adapted from Ancona and Caldwell (1992) capturing individual team member boundary-spanning behaviors across client, faculty advisor, and external organizational interfaces.</t>
+        </is>
+      </c>
+      <c r="AH25" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI25" t="n">
+        <v>999</v>
+      </c>
+      <c r="AJ25" t="n">
+        <v>999</v>
+      </c>
+      <c r="AK25" t="inlineStr">
+        <is>
+          <t>4 = Objective / Sociometric</t>
+        </is>
+      </c>
+      <c r="AL25" t="inlineStr">
+        <is>
+          <t>Continuous standardized test score</t>
+        </is>
+      </c>
+      <c r="AM25" t="inlineStr">
+        <is>
+          <t>GMAT score</t>
+        </is>
+      </c>
+      <c r="AN25" t="inlineStr">
+        <is>
+          <t>Continuous Graduate Management Admission Test (GMAT) cognitive ability score used as an individual control variable.</t>
+        </is>
+      </c>
+      <c r="AO25" t="inlineStr">
+        <is>
+          <t>Boundary-spanning behavior</t>
+        </is>
+      </c>
+      <c r="AP25" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AQ25" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AR25" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AS25" t="inlineStr">
+        <is>
+          <t>GMAT score</t>
+        </is>
+      </c>
+      <c r="AT25" t="n">
+        <v>653.9</v>
+      </c>
+      <c r="AU25" t="n">
+        <v>57.89</v>
+      </c>
+      <c r="AV25" t="n">
+        <v>999</v>
+      </c>
+      <c r="AW25" t="n">
+        <v>-0.19</v>
+      </c>
+      <c r="AX25" t="inlineStr">
+        <is>
+          <t>Table 1 (p. 1432) | Row: "5. GMAT score" x Col: "1. Boundary-spanning behavior" = -.19* | Pairwise n = 177 (Total N = 190) | Table Footnote: "* p &lt; .05 ** p &lt; .01"</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>399</v>
+      </c>
+      <c r="D26" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>1 = include</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>1 = Cross-sectional design</t>
+        </is>
+      </c>
+      <c r="S26" t="inlineStr">
+        <is>
+          <t>United States</t>
+        </is>
+      </c>
+      <c r="T26" t="inlineStr">
+        <is>
+          <t>Mid-Atlantic United States</t>
+        </is>
+      </c>
+      <c r="U26" t="inlineStr">
+        <is>
+          <t>0 = Domestic</t>
+        </is>
+      </c>
+      <c r="V26" t="n">
+        <v>190</v>
+      </c>
+      <c r="W26" t="n">
+        <v>999</v>
+      </c>
+      <c r="X26" t="n">
+        <v>999</v>
+      </c>
+      <c r="Y26" t="n">
+        <v>999</v>
+      </c>
+      <c r="Z26" t="inlineStr">
+        <is>
+          <t>MBA students (consulting teams)</t>
+        </is>
+      </c>
+      <c r="AA26" t="n">
+        <v>6</v>
+      </c>
+      <c r="AB26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AC26" t="n">
+        <v>5</v>
+      </c>
+      <c r="AD26" t="inlineStr">
+        <is>
+          <t>2 = Peer-report</t>
+        </is>
+      </c>
+      <c r="AE26" t="inlineStr">
+        <is>
+          <t>Peer ratings across consulting teammates justified by median rwg = 0.80, ICC(1) = 0.28, ICC(2) = 0.71.</t>
+        </is>
+      </c>
+      <c r="AF26" t="inlineStr">
+        <is>
+          <t>Ancona and Caldwell's (1992)</t>
+        </is>
+      </c>
+      <c r="AG26" t="inlineStr">
+        <is>
+          <t>Six items adapted from Ancona and Caldwell (1992) capturing individual team member boundary-spanning behaviors across client, faculty advisor, and external organizational interfaces.</t>
+        </is>
+      </c>
+      <c r="AH26" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI26" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ26" t="n">
+        <v>5</v>
+      </c>
+      <c r="AK26" t="inlineStr">
+        <is>
+          <t>1 = Self-report</t>
+        </is>
+      </c>
+      <c r="AM26" t="inlineStr">
+        <is>
+          <t>Beehr et al. (1976)</t>
+        </is>
+      </c>
+      <c r="AN26" t="inlineStr">
+        <is>
+          <t>Three-item role overload scale adapted from Beehr et al. (1976) rated on a 5-point Likert scale (alpha = 0.83).</t>
+        </is>
+      </c>
+      <c r="AO26" t="inlineStr">
+        <is>
+          <t>Boundary-spanning behavior</t>
+        </is>
+      </c>
+      <c r="AP26" t="n">
+        <v>2.91</v>
+      </c>
+      <c r="AQ26" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="AR26" t="n">
+        <v>0.86</v>
+      </c>
+      <c r="AS26" t="inlineStr">
+        <is>
+          <t>Role overload</t>
+        </is>
+      </c>
+      <c r="AT26" t="n">
+        <v>2.47</v>
+      </c>
+      <c r="AU26" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="AV26" t="n">
+        <v>0.83</v>
+      </c>
+      <c r="AW26" t="n">
+        <v>-0.04</v>
+      </c>
+      <c r="AX26" t="inlineStr">
+        <is>
+          <t>Table 1 (p. 1432) | Row: "6. Role overload" x Col: "1. Boundary-spanning behavior" = -.04 | Pairwise n = 186 (Total N = 190) | Table Footnote: "* p &lt; .05 ** p &lt; .01"</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>403</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>0 = exclude</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>3 = Non-individual level (team/firm/org analysis)</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>The unit of statistical analysis is the business organization (N = 62 publicly held U.S. corporations on the Russell 1000 index). The 62 Public Affairs Managers served merely as single key informants evaluating the firm's macro-level relationships with public interest groups using firm-referent items (e.g., The firm avoids close contact with this socio-political actor), violating Screening Rule 4 and Rule 5 (Proxy Guardrail). Verbatim Evidence: [p. 58] "A survey of 62 Public Affairs Managers in publicly held U.S. corporations finds that organizations adopt relational styles similar to those theorized in studies of inter-organizational conflict, organizational communication and stakeholder management." [p. 62] "The organizations participating in this study were large, U.S. companies listed on the Russell 1000 index from a variety of industries... A limitation of the study is that only one manager responded for each organization. The vulnerability inherent in this practice is that the manager's understanding reflected in the survey may not be representative of the organization's practices."</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>KY</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
         <v>407</v>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E28" t="inlineStr">
         <is>
           <t>0 = exclude</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F28" t="inlineStr">
         <is>
           <t>1 = No effect size of interest</t>
         </is>
       </c>
-      <c r="P24" t="inlineStr">
+      <c r="P28" t="inlineStr">
         <is>
           <t>The study surveys 193 county human service managers across five San Francisco Bay Area departments and measures managerial boundary spanning, but reports NO bivariate zero-order Pearson correlation matrix (r) involving boundary spanning. The only statistical results reported are multivariate ordinal logistic regressions with odds ratios (Table 4). Under Screening Rule 7, studies lacking extractable bivariate zero-order effect sizes must be excluded under Code 1. Verbatim Evidence: [p. 115] "A 2015 survey of 193 managers from five San Francisco Bay Area county human service departments examined the relationship between contract-based service coordination... and the predictors of managerial role, involvement, and boundary spanning. Multivariate regression results suggested that county managers identified fewer service coordination challenges if they were at the executive and program levels, had greater contract involvement, and engaged in contract-focused boundary spanning." [p. 122] "Bivariate Pearson, Spearman, and phi correlation tests did not indicate any problematic collinearity among independent variables (e.g., &gt; 0.33). Nor were the dependent variables highly correlated with any of the independent or control variables (i.e., all &gt; 0.21)."</t>
         </is>

</xml_diff>

<commit_message>
fix(reverify): 100% exhaustive PDF re-verification across batches 392-407 and 501-511
</commit_message>
<xml_diff>
--- a/03_Coding_Sheets/392_398_399_403_407.xlsx
+++ b/03_Coding_Sheets/392_398_399_403_407.xlsx
@@ -778,7 +778,7 @@
       </c>
       <c r="AE4" t="inlineStr">
         <is>
-          <t>Sociometric outdegree centrality metric computed as the number of communication contacts initiated with other organization members in the internal network.</t>
+          <t>Sociometric roster tie count of direct internal communication contacts initiated by the manager (Rule 28 internal dissemination step).</t>
         </is>
       </c>
       <c r="AF4" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="AG4" t="inlineStr">
         <is>
-          <t>Internal communication outdegree operationalizing the internal information dissemination/transfer step of the two-step boundary-spanning information processing model (Tushman &amp; Scanlan, 1981; Rule 28).</t>
+          <t>Centrality, which is the most important network indicator of structural location at the individual level, is measured by outdegree (Freeman, 1979). Outdegree stands for the number of direct contacts that an individual initiates and therefore measures potential communication activity. It is measured in both the internal and extended networks of the sample organization.</t>
         </is>
       </c>
       <c r="AH4" t="n">
@@ -812,7 +812,7 @@
       </c>
       <c r="AN4" t="inlineStr">
         <is>
-          <t>Three-level hierarchical management status coded as top, middle, and lower management (1 = lower management, 3 = top management).</t>
+          <t>Hierarchical level reflects the three existing major levels of management in the organization and is measured as top, middle, and lower management.</t>
         </is>
       </c>
       <c r="AO4" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="AX4" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "2. Outdegree in internal network" x Col: "1. Hierarchical level" = .26 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "2. Outdegree in internal network" x Col: "1. Hierarchical level" = .26 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -922,7 +922,7 @@
       </c>
       <c r="AE5" t="inlineStr">
         <is>
-          <t>Sociometric name generator instructing the respondent to list individuals with whom he/she communicated to get the job done outside the organization.</t>
+          <t>Sociometric count of direct external communication contacts outside the organization (vendors, contractors, regulatory and transit agencies).</t>
         </is>
       </c>
       <c r="AF5" t="inlineStr">
@@ -932,7 +932,7 @@
       </c>
       <c r="AG5" t="inlineStr">
         <is>
-          <t>Individual boundary-spanning ties measuring direct external communication contacts with members of outside organizations (vendors, contractors, regulatory and transit agencies).</t>
+          <t>The survey asked questions about background characteristics, followed by a sociometric instrument that instructed the respondent to list individuals with whom he/she communicated "to get the job done" both within and outside the organization.</t>
         </is>
       </c>
       <c r="AH5" t="n">
@@ -956,7 +956,7 @@
       </c>
       <c r="AN5" t="inlineStr">
         <is>
-          <t>Three-level hierarchical management status coded as top, middle, and lower management (1 = lower management, 3 = top management).</t>
+          <t>Hierarchical level reflects the three existing major levels of management in the organization and is measured as top, middle, and lower management.</t>
         </is>
       </c>
       <c r="AO5" t="inlineStr">
@@ -992,7 +992,7 @@
       </c>
       <c r="AX5" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "3. Boundary spanning ties" x Col: "1. Hierarchical level" = .32 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "3. Boundary spanning ties" x Col: "1. Hierarchical level" = .32 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -1066,7 +1066,7 @@
       </c>
       <c r="AE6" t="inlineStr">
         <is>
-          <t>Sociometric outdegree centrality metric computed as the total number of communication contacts initiated across both internal and external network ties.</t>
+          <t>Sociometric count of total communication contacts across both internal organization members and external boundary-spanning contacts.</t>
         </is>
       </c>
       <c r="AF6" t="inlineStr">
@@ -1076,7 +1076,7 @@
       </c>
       <c r="AG6" t="inlineStr">
         <is>
-          <t>Centrality in the extended organizational network measuring total communication contacts across both internal core members and external boundary-spanning partners (Freeman, 1979).</t>
+          <t>Centrality, which is the most important network indicator of structural location at the individual level, is measured by outdegree (Freeman, 1979). Outdegree stands for the number of direct contacts that an individual initiates and therefore measures potential communication activity. It is measured in both the internal and extended networks of the sample organization.</t>
         </is>
       </c>
       <c r="AH6" t="n">
@@ -1100,7 +1100,7 @@
       </c>
       <c r="AN6" t="inlineStr">
         <is>
-          <t>Three-level hierarchical management status coded as top, middle, and lower management (1 = lower management, 3 = top management).</t>
+          <t>Hierarchical level reflects the three existing major levels of management in the organization and is measured as top, middle, and lower management.</t>
         </is>
       </c>
       <c r="AO6" t="inlineStr">
@@ -1136,7 +1136,7 @@
       </c>
       <c r="AX6" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "4. Outdegree in extended network" x Col: "1. Hierarchical level" = .35 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "4. Outdegree in extended network" x Col: "1. Hierarchical level" = .35 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -1210,17 +1210,17 @@
       </c>
       <c r="AE7" t="inlineStr">
         <is>
-          <t>Relative external boundary-spanning orientation calculated as the ratio of boundary-spanning ties divided by total ties (external plus internal).</t>
+          <t>Proportion of boundary-spanning ties divided by total ties (external plus internal) in the extended network.</t>
         </is>
       </c>
       <c r="AF7" t="inlineStr">
         <is>
-          <t>orientation of an individual's network</t>
+          <t>number of boundary-spanning ties divided by the total number of ties (external plus internal)</t>
         </is>
       </c>
       <c r="AG7" t="inlineStr">
         <is>
-          <t>Network orientation index measuring the proportion of boundary-spanning ties relative to total communication ties in the extended network.</t>
+          <t>As earlier defined, the orientation of an individual's network is the number of boundary-spanning ties divided by the total number of ties (external plus internal). A high value (up to 1) stands for external orientation, whereas a zero score indicates an entirely internal orientation.</t>
         </is>
       </c>
       <c r="AH7" t="n">
@@ -1244,7 +1244,7 @@
       </c>
       <c r="AN7" t="inlineStr">
         <is>
-          <t>Three-level hierarchical management status coded as top, middle, and lower management (1 = lower management, 3 = top management).</t>
+          <t>Hierarchical level reflects the three existing major levels of management in the organization and is measured as top, middle, and lower management.</t>
         </is>
       </c>
       <c r="AO7" t="inlineStr">
@@ -1280,7 +1280,7 @@
       </c>
       <c r="AX7" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "5. Boundary spanning orientation" x Col: "1. Hierarchical level" = .15 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "5. Boundary spanning orientation" x Col: "1. Hierarchical level" = .15 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -1354,7 +1354,7 @@
       </c>
       <c r="AE8" t="inlineStr">
         <is>
-          <t>Sociometric outdegree centrality metric computed as the number of communication contacts initiated with other organization members in the internal network.</t>
+          <t>Sociometric roster tie count of direct internal communication contacts initiated by the manager (Rule 28 internal dissemination step).</t>
         </is>
       </c>
       <c r="AF8" t="inlineStr">
@@ -1364,7 +1364,7 @@
       </c>
       <c r="AG8" t="inlineStr">
         <is>
-          <t>Internal communication outdegree operationalizing the internal information dissemination/transfer step of the two-step boundary-spanning information processing model (Tushman &amp; Scanlan, 1981; Rule 28).</t>
+          <t>Centrality, which is the most important network indicator of structural location at the individual level, is measured by outdegree (Freeman, 1979). Outdegree stands for the number of direct contacts that an individual initiates and therefore measures potential communication activity. It is measured in both the internal and extended networks of the sample organization.</t>
         </is>
       </c>
       <c r="AH8" t="n">
@@ -1388,7 +1388,7 @@
       </c>
       <c r="AN8" t="inlineStr">
         <is>
-          <t>Five-item self-perceived decision-making influence scale adapted from Van de Ven and Ferry (1980) on a 5-point scale (1 = none to 5 = very much; alpha = 0.91).</t>
+          <t>Individual influence is measured by two variables. The first one, suggested by Van de Ven and Ferry (1980), measures self-perceived influence in decision making. It is computed as the sum of the responses (on a 5-point scale) to questions about the influence the respondent has over determining the goals for the work unit, policies and procedures, and decisions about hiring, promotion, and salary increases (Cronbach's alpha = .91).</t>
         </is>
       </c>
       <c r="AO8" t="inlineStr">
@@ -1424,7 +1424,7 @@
       </c>
       <c r="AX8" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "2. Outdegree in internal network" = .35 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "2. Outdegree in internal network" = .35 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="AE9" t="inlineStr">
         <is>
-          <t>Sociometric name generator instructing the respondent to list individuals with whom he/she communicated to get the job done outside the organization.</t>
+          <t>Sociometric count of direct external communication contacts outside the organization (vendors, contractors, regulatory and transit agencies).</t>
         </is>
       </c>
       <c r="AF9" t="inlineStr">
@@ -1508,7 +1508,7 @@
       </c>
       <c r="AG9" t="inlineStr">
         <is>
-          <t>Individual boundary-spanning ties measuring direct external communication contacts with members of outside organizations (vendors, contractors, regulatory and transit agencies).</t>
+          <t>The survey asked questions about background characteristics, followed by a sociometric instrument that instructed the respondent to list individuals with whom he/she communicated "to get the job done" both within and outside the organization.</t>
         </is>
       </c>
       <c r="AH9" t="n">
@@ -1532,7 +1532,7 @@
       </c>
       <c r="AN9" t="inlineStr">
         <is>
-          <t>Five-item self-perceived decision-making influence scale adapted from Van de Ven and Ferry (1980) on a 5-point scale (1 = none to 5 = very much; alpha = 0.91).</t>
+          <t>Individual influence is measured by two variables. The first one, suggested by Van de Ven and Ferry (1980), measures self-perceived influence in decision making. It is computed as the sum of the responses (on a 5-point scale) to questions about the influence the respondent has over determining the goals for the work unit, policies and procedures, and decisions about hiring, promotion, and salary increases (Cronbach's alpha = .91).</t>
         </is>
       </c>
       <c r="AO9" t="inlineStr">
@@ -1568,7 +1568,7 @@
       </c>
       <c r="AX9" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "3. Boundary spanning ties" = .34 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "3. Boundary spanning ties" = .34 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -1642,7 +1642,7 @@
       </c>
       <c r="AE10" t="inlineStr">
         <is>
-          <t>Sociometric outdegree centrality metric computed as the total number of communication contacts initiated across both internal and external network ties.</t>
+          <t>Sociometric count of total communication contacts across both internal organization members and external boundary-spanning contacts.</t>
         </is>
       </c>
       <c r="AF10" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="AG10" t="inlineStr">
         <is>
-          <t>Centrality in the extended organizational network measuring total communication contacts across both internal core members and external boundary-spanning partners (Freeman, 1979).</t>
+          <t>Centrality, which is the most important network indicator of structural location at the individual level, is measured by outdegree (Freeman, 1979). Outdegree stands for the number of direct contacts that an individual initiates and therefore measures potential communication activity. It is measured in both the internal and extended networks of the sample organization.</t>
         </is>
       </c>
       <c r="AH10" t="n">
@@ -1676,7 +1676,7 @@
       </c>
       <c r="AN10" t="inlineStr">
         <is>
-          <t>Five-item self-perceived decision-making influence scale adapted from Van de Ven and Ferry (1980) on a 5-point scale (1 = none to 5 = very much; alpha = 0.91).</t>
+          <t>Individual influence is measured by two variables. The first one, suggested by Van de Ven and Ferry (1980), measures self-perceived influence in decision making. It is computed as the sum of the responses (on a 5-point scale) to questions about the influence the respondent has over determining the goals for the work unit, policies and procedures, and decisions about hiring, promotion, and salary increases (Cronbach's alpha = .91).</t>
         </is>
       </c>
       <c r="AO10" t="inlineStr">
@@ -1708,11 +1708,11 @@
         <v>0.91</v>
       </c>
       <c r="AW10" t="n">
-        <v>0.4</v>
+        <v>0.42</v>
       </c>
       <c r="AX10" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "4. Outdegree in extended network" = .40 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "4. Outdegree in extended network" = .42 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -1786,17 +1786,17 @@
       </c>
       <c r="AE11" t="inlineStr">
         <is>
-          <t>Relative external boundary-spanning orientation calculated as the ratio of boundary-spanning ties divided by total ties (external plus internal).</t>
+          <t>Proportion of boundary-spanning ties divided by total ties (external plus internal) in the extended network.</t>
         </is>
       </c>
       <c r="AF11" t="inlineStr">
         <is>
-          <t>orientation of an individual's network</t>
+          <t>number of boundary-spanning ties divided by the total number of ties (external plus internal)</t>
         </is>
       </c>
       <c r="AG11" t="inlineStr">
         <is>
-          <t>Network orientation index measuring the proportion of boundary-spanning ties relative to total communication ties in the extended network.</t>
+          <t>As earlier defined, the orientation of an individual's network is the number of boundary-spanning ties divided by the total number of ties (external plus internal). A high value (up to 1) stands for external orientation, whereas a zero score indicates an entirely internal orientation.</t>
         </is>
       </c>
       <c r="AH11" t="n">
@@ -1820,7 +1820,7 @@
       </c>
       <c r="AN11" t="inlineStr">
         <is>
-          <t>Five-item self-perceived decision-making influence scale adapted from Van de Ven and Ferry (1980) on a 5-point scale (1 = none to 5 = very much; alpha = 0.91).</t>
+          <t>Individual influence is measured by two variables. The first one, suggested by Van de Ven and Ferry (1980), measures self-perceived influence in decision making. It is computed as the sum of the responses (on a 5-point scale) to questions about the influence the respondent has over determining the goals for the work unit, policies and procedures, and decisions about hiring, promotion, and salary increases (Cronbach's alpha = .91).</t>
         </is>
       </c>
       <c r="AO11" t="inlineStr">
@@ -1852,11 +1852,11 @@
         <v>0.91</v>
       </c>
       <c r="AW11" t="n">
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="AX11" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "5. Boundary spanning orientation" = .16 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "6. Self-perceived influence" x Col: "5. Boundary spanning orientation" = .14 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="AE12" t="inlineStr">
         <is>
-          <t>Sociometric outdegree centrality metric computed as the number of communication contacts initiated with other organization members in the internal network.</t>
+          <t>Sociometric roster tie count of direct internal communication contacts initiated by the manager (Rule 28 internal dissemination step).</t>
         </is>
       </c>
       <c r="AF12" t="inlineStr">
@@ -1940,7 +1940,7 @@
       </c>
       <c r="AG12" t="inlineStr">
         <is>
-          <t>Internal communication outdegree operationalizing the internal information dissemination/transfer step of the two-step boundary-spanning information processing model (Tushman &amp; Scanlan, 1981; Rule 28).</t>
+          <t>Centrality, which is the most important network indicator of structural location at the individual level, is measured by outdegree (Freeman, 1979). Outdegree stands for the number of direct contacts that an individual initiates and therefore measures potential communication activity. It is measured in both the internal and extended networks of the sample organization.</t>
         </is>
       </c>
       <c r="AH12" t="n">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="AL12" t="inlineStr">
         <is>
-          <t>Sociometric peer rating where each communicating alter rates ego's influence on a 1-5 scale, summed across alters.</t>
+          <t>Sociometric peer-attributed influence ratings summed across alters.</t>
         </is>
       </c>
       <c r="AM12" t="inlineStr">
@@ -1969,7 +1969,7 @@
       </c>
       <c r="AN12" t="inlineStr">
         <is>
-          <t>Single-item sociometric peer-attributed influence rating summed across all alters with whom the respondent communicated (1 = none at all to 5 = a great deal).</t>
+          <t>Since self-perceived indicators may be biased, a second measure of influence is added-attributed influence. It measures the influence that other organization members attribute to the respondent. To calculate it, we asked respondents, or egos in network terms, to rate how much influence every manager with whom they communicated (alter) had on their work performance. These ratings were then summed for every alter, and these sums measure attributed influence.</t>
         </is>
       </c>
       <c r="AO12" t="inlineStr">
@@ -2001,11 +2001,11 @@
         <v>999</v>
       </c>
       <c r="AW12" t="n">
-        <v>0.58</v>
+        <v>0.32</v>
       </c>
       <c r="AX12" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "2. Outdegree in internal network" = .58 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "2. Outdegree in internal network" = .32 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2079,7 @@
       </c>
       <c r="AE13" t="inlineStr">
         <is>
-          <t>Sociometric name generator instructing the respondent to list individuals with whom he/she communicated to get the job done outside the organization.</t>
+          <t>Sociometric count of direct external communication contacts outside the organization (vendors, contractors, regulatory and transit agencies).</t>
         </is>
       </c>
       <c r="AF13" t="inlineStr">
@@ -2089,7 +2089,7 @@
       </c>
       <c r="AG13" t="inlineStr">
         <is>
-          <t>Individual boundary-spanning ties measuring direct external communication contacts with members of outside organizations (vendors, contractors, regulatory and transit agencies).</t>
+          <t>The survey asked questions about background characteristics, followed by a sociometric instrument that instructed the respondent to list individuals with whom he/she communicated "to get the job done" both within and outside the organization.</t>
         </is>
       </c>
       <c r="AH13" t="n">
@@ -2108,7 +2108,7 @@
       </c>
       <c r="AL13" t="inlineStr">
         <is>
-          <t>Sociometric peer rating where each communicating alter rates ego's influence on a 1-5 scale, summed across alters.</t>
+          <t>Sociometric peer-attributed influence ratings summed across alters.</t>
         </is>
       </c>
       <c r="AM13" t="inlineStr">
@@ -2118,7 +2118,7 @@
       </c>
       <c r="AN13" t="inlineStr">
         <is>
-          <t>Single-item sociometric peer-attributed influence rating summed across all alters with whom the respondent communicated (1 = none at all to 5 = a great deal).</t>
+          <t>Since self-perceived indicators may be biased, a second measure of influence is added-attributed influence. It measures the influence that other organization members attribute to the respondent. To calculate it, we asked respondents, or egos in network terms, to rate how much influence every manager with whom they communicated (alter) had on their work performance. These ratings were then summed for every alter, and these sums measure attributed influence.</t>
         </is>
       </c>
       <c r="AO13" t="inlineStr">
@@ -2150,11 +2150,11 @@
         <v>999</v>
       </c>
       <c r="AW13" t="n">
-        <v>0.51</v>
+        <v>0.32</v>
       </c>
       <c r="AX13" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "3. Boundary spanning ties" = .51 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "3. Boundary spanning ties" = .32 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -2228,7 +2228,7 @@
       </c>
       <c r="AE14" t="inlineStr">
         <is>
-          <t>Sociometric outdegree centrality metric computed as the total number of communication contacts initiated across both internal and external network ties.</t>
+          <t>Sociometric count of total communication contacts across both internal organization members and external boundary-spanning contacts.</t>
         </is>
       </c>
       <c r="AF14" t="inlineStr">
@@ -2238,7 +2238,7 @@
       </c>
       <c r="AG14" t="inlineStr">
         <is>
-          <t>Centrality in the extended organizational network measuring total communication contacts across both internal core members and external boundary-spanning partners (Freeman, 1979).</t>
+          <t>Centrality, which is the most important network indicator of structural location at the individual level, is measured by outdegree (Freeman, 1979). Outdegree stands for the number of direct contacts that an individual initiates and therefore measures potential communication activity. It is measured in both the internal and extended networks of the sample organization.</t>
         </is>
       </c>
       <c r="AH14" t="n">
@@ -2257,7 +2257,7 @@
       </c>
       <c r="AL14" t="inlineStr">
         <is>
-          <t>Sociometric peer rating where each communicating alter rates ego's influence on a 1-5 scale, summed across alters.</t>
+          <t>Sociometric peer-attributed influence ratings summed across alters.</t>
         </is>
       </c>
       <c r="AM14" t="inlineStr">
@@ -2267,7 +2267,7 @@
       </c>
       <c r="AN14" t="inlineStr">
         <is>
-          <t>Single-item sociometric peer-attributed influence rating summed across all alters with whom the respondent communicated (1 = none at all to 5 = a great deal).</t>
+          <t>Since self-perceived indicators may be biased, a second measure of influence is added-attributed influence. It measures the influence that other organization members attribute to the respondent. To calculate it, we asked respondents, or egos in network terms, to rate how much influence every manager with whom they communicated (alter) had on their work performance. These ratings were then summed for every alter, and these sums measure attributed influence.</t>
         </is>
       </c>
       <c r="AO14" t="inlineStr">
@@ -2299,11 +2299,11 @@
         <v>999</v>
       </c>
       <c r="AW14" t="n">
-        <v>0.63</v>
+        <v>0.39</v>
       </c>
       <c r="AX14" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "4. Outdegree in extended network" = .63 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "4. Outdegree in extended network" = .39 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -2377,17 +2377,17 @@
       </c>
       <c r="AE15" t="inlineStr">
         <is>
-          <t>Relative external boundary-spanning orientation calculated as the ratio of boundary-spanning ties divided by total ties (external plus internal).</t>
+          <t>Proportion of boundary-spanning ties divided by total ties (external plus internal) in the extended network.</t>
         </is>
       </c>
       <c r="AF15" t="inlineStr">
         <is>
-          <t>orientation of an individual's network</t>
+          <t>number of boundary-spanning ties divided by the total number of ties (external plus internal)</t>
         </is>
       </c>
       <c r="AG15" t="inlineStr">
         <is>
-          <t>Network orientation index measuring the proportion of boundary-spanning ties relative to total communication ties in the extended network.</t>
+          <t>As earlier defined, the orientation of an individual's network is the number of boundary-spanning ties divided by the total number of ties (external plus internal). A high value (up to 1) stands for external orientation, whereas a zero score indicates an entirely internal orientation.</t>
         </is>
       </c>
       <c r="AH15" t="n">
@@ -2406,7 +2406,7 @@
       </c>
       <c r="AL15" t="inlineStr">
         <is>
-          <t>Sociometric peer rating where each communicating alter rates ego's influence on a 1-5 scale, summed across alters.</t>
+          <t>Sociometric peer-attributed influence ratings summed across alters.</t>
         </is>
       </c>
       <c r="AM15" t="inlineStr">
@@ -2416,7 +2416,7 @@
       </c>
       <c r="AN15" t="inlineStr">
         <is>
-          <t>Single-item sociometric peer-attributed influence rating summed across all alters with whom the respondent communicated (1 = none at all to 5 = a great deal).</t>
+          <t>Since self-perceived indicators may be biased, a second measure of influence is added-attributed influence. It measures the influence that other organization members attribute to the respondent. To calculate it, we asked respondents, or egos in network terms, to rate how much influence every manager with whom they communicated (alter) had on their work performance. These ratings were then summed for every alter, and these sums measure attributed influence.</t>
         </is>
       </c>
       <c r="AO15" t="inlineStr">
@@ -2448,11 +2448,11 @@
         <v>999</v>
       </c>
       <c r="AW15" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="AX15" t="inlineStr">
         <is>
-          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "5. Boundary spanning orientation" = .17 | Listwise N = 108 | Table Footnote: "N = 108. All correlations are significant at p &lt; .05, except for .15 and .16, which are significant at p &lt; .10."</t>
+          <t>Table 1 (p. 194) | Row: "7. Attributed influence" x Col: "5. Boundary spanning orientation" = .15 | Listwise N = 108 | Table Footnote: "Note. Correlations above .20 are significant at .05 level."</t>
         </is>
       </c>
     </row>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="Q16" t="inlineStr">
         <is>
-          <t>1 = Cross-sectional design</t>
+          <t>2 = Longitudinal design</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -2492,21 +2492,21 @@
         <v>170</v>
       </c>
       <c r="W16" t="n">
-        <v>39</v>
+        <v>41.92</v>
       </c>
       <c r="X16" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="Y16" t="n">
-        <v>6</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="Z16" t="inlineStr">
         <is>
-          <t>Engineers / Engineering employees</t>
+          <t>Employees in a manufacturing and engineering firm (nonmanagement team members)</t>
         </is>
       </c>
       <c r="AA16" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="AB16" t="n">
         <v>1</v>
@@ -2521,12 +2521,12 @@
       </c>
       <c r="AF16" t="inlineStr">
         <is>
-          <t>Marrone et al., 2007</t>
+          <t>Ancona and Caldwell’s (1992)</t>
         </is>
       </c>
       <c r="AG16" t="inlineStr">
         <is>
-          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
+          <t>We closely followed Ancona and Caldwell’s (1992) development of boundary-spanning items and selected 13 items from their research to assess the extent to which team members engaged in various boundary-spanning behaviors aimed at establishing and maintaining relationships with key external parties. Two of our constructs, supportive coaching and boundary-spanning self-efficacy, used traditional Likert scales (1 = strongly disagree to 5 = strongly agree), whereas our other two constructs utilized alternative anchor points (boundary spanning behavior, 1 = a very small extent to 5 = a very great extent; job satisfaction, 1 = very dissatisfied to 5 = very satisfied).</t>
         </is>
       </c>
       <c r="AH16" t="n">
@@ -2545,12 +2545,12 @@
       </c>
       <c r="AM16" t="inlineStr">
         <is>
-          <t>demographic question</t>
+          <t>measured age in years</t>
         </is>
       </c>
       <c r="AN16" t="inlineStr">
         <is>
-          <t>Participant age in years measured as a continuous demographic variable.</t>
+          <t>We included gender, age, and ethnicity/race as variables in all substantive equations. We measured age in years; we coded gender using male = 1 and female = 2.</t>
         </is>
       </c>
       <c r="AO16" t="inlineStr">
@@ -2559,13 +2559,13 @@
         </is>
       </c>
       <c r="AP16" t="n">
-        <v>3.48</v>
+        <v>2.62</v>
       </c>
       <c r="AQ16" t="n">
-        <v>0.65</v>
+        <v>0.83</v>
       </c>
       <c r="AR16" t="n">
-        <v>0.88</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AS16" t="inlineStr">
         <is>
@@ -2573,10 +2573,10 @@
         </is>
       </c>
       <c r="AT16" t="n">
-        <v>39</v>
+        <v>41.92</v>
       </c>
       <c r="AU16" t="n">
-        <v>12</v>
+        <v>11.11</v>
       </c>
       <c r="AV16" t="n">
         <v>999</v>
@@ -2609,7 +2609,7 @@
       </c>
       <c r="Q17" t="inlineStr">
         <is>
-          <t>1 = Cross-sectional design</t>
+          <t>2 = Longitudinal design</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2626,21 +2626,21 @@
         <v>170</v>
       </c>
       <c r="W17" t="n">
-        <v>39</v>
+        <v>41.92</v>
       </c>
       <c r="X17" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="Y17" t="n">
-        <v>6</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="Z17" t="inlineStr">
         <is>
-          <t>Engineers / Engineering employees</t>
+          <t>Employees in a manufacturing and engineering firm (nonmanagement team members)</t>
         </is>
       </c>
       <c r="AA17" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="AB17" t="n">
         <v>1</v>
@@ -2655,12 +2655,12 @@
       </c>
       <c r="AF17" t="inlineStr">
         <is>
-          <t>Marrone et al., 2007</t>
+          <t>Ancona and Caldwell’s (1992)</t>
         </is>
       </c>
       <c r="AG17" t="inlineStr">
         <is>
-          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
+          <t>We closely followed Ancona and Caldwell’s (1992) development of boundary-spanning items and selected 13 items from their research to assess the extent to which team members engaged in various boundary-spanning behaviors aimed at establishing and maintaining relationships with key external parties. Two of our constructs, supportive coaching and boundary-spanning self-efficacy, used traditional Likert scales (1 = strongly disagree to 5 = strongly agree), whereas our other two constructs utilized alternative anchor points (boundary spanning behavior, 1 = a very small extent to 5 = a very great extent; job satisfaction, 1 = very dissatisfied to 5 = very satisfied).</t>
         </is>
       </c>
       <c r="AH17" t="n">
@@ -2679,12 +2679,12 @@
       </c>
       <c r="AM17" t="inlineStr">
         <is>
-          <t>demographic question</t>
+          <t>coded gender using male = 1 and female = 2</t>
         </is>
       </c>
       <c r="AN17" t="inlineStr">
         <is>
-          <t>Participant gender coded as female = 1 and male = 2.</t>
+          <t>We included gender, age, and ethnicity/race as variables in all substantive equations. We measured age in years; we coded gender using male = 1 and female = 2.</t>
         </is>
       </c>
       <c r="AO17" t="inlineStr">
@@ -2693,13 +2693,13 @@
         </is>
       </c>
       <c r="AP17" t="n">
-        <v>3.48</v>
+        <v>2.62</v>
       </c>
       <c r="AQ17" t="n">
-        <v>0.65</v>
+        <v>0.83</v>
       </c>
       <c r="AR17" t="n">
-        <v>0.88</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AS17" t="inlineStr">
         <is>
@@ -2707,10 +2707,10 @@
         </is>
       </c>
       <c r="AT17" t="n">
-        <v>1.79</v>
+        <v>1.1</v>
       </c>
       <c r="AU17" t="n">
-        <v>0.41</v>
+        <v>0.3</v>
       </c>
       <c r="AV17" t="n">
         <v>999</v>
@@ -2743,7 +2743,7 @@
       </c>
       <c r="Q18" t="inlineStr">
         <is>
-          <t>1 = Cross-sectional design</t>
+          <t>2 = Longitudinal design</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2760,21 +2760,21 @@
         <v>170</v>
       </c>
       <c r="W18" t="n">
-        <v>39</v>
+        <v>41.92</v>
       </c>
       <c r="X18" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="Y18" t="n">
-        <v>6</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="Z18" t="inlineStr">
         <is>
-          <t>Engineers / Engineering employees</t>
+          <t>Employees in a manufacturing and engineering firm (nonmanagement team members)</t>
         </is>
       </c>
       <c r="AA18" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="AB18" t="n">
         <v>1</v>
@@ -2789,12 +2789,12 @@
       </c>
       <c r="AF18" t="inlineStr">
         <is>
-          <t>Marrone et al., 2007</t>
+          <t>Ancona and Caldwell’s (1992)</t>
         </is>
       </c>
       <c r="AG18" t="inlineStr">
         <is>
-          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
+          <t>We closely followed Ancona and Caldwell’s (1992) development of boundary-spanning items and selected 13 items from their research to assess the extent to which team members engaged in various boundary-spanning behaviors aimed at establishing and maintaining relationships with key external parties. Two of our constructs, supportive coaching and boundary-spanning self-efficacy, used traditional Likert scales (1 = strongly disagree to 5 = strongly agree), whereas our other two constructs utilized alternative anchor points (boundary spanning behavior, 1 = a very small extent to 5 = a very great extent; job satisfaction, 1 = very dissatisfied to 5 = very satisfied).</t>
         </is>
       </c>
       <c r="AH18" t="n">
@@ -2813,12 +2813,12 @@
       </c>
       <c r="AM18" t="inlineStr">
         <is>
-          <t>demographic question</t>
+          <t>coded the measure using Caucasian/White = 1 and all others = 2</t>
         </is>
       </c>
       <c r="AN18" t="inlineStr">
         <is>
-          <t>Ethnicity/race coded as Caucasian/White = 1 and all others = 2.</t>
+          <t>Finally, we asked respondents, “What is your ethnicity/race?” and included seven response options: African American/Black, Asian, Caucasian/White, Hispanic/Latino, Native American, Pacific Islander, and Other. Given the preponderance of Caucasian/White respondents, we ultimately coded the measure using Caucasian/White = 1 and all others = 2.</t>
         </is>
       </c>
       <c r="AO18" t="inlineStr">
@@ -2827,13 +2827,13 @@
         </is>
       </c>
       <c r="AP18" t="n">
-        <v>3.48</v>
+        <v>2.62</v>
       </c>
       <c r="AQ18" t="n">
-        <v>0.65</v>
+        <v>0.83</v>
       </c>
       <c r="AR18" t="n">
-        <v>0.88</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AS18" t="inlineStr">
         <is>
@@ -2877,7 +2877,7 @@
       </c>
       <c r="Q19" t="inlineStr">
         <is>
-          <t>1 = Cross-sectional design</t>
+          <t>2 = Longitudinal design</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2894,21 +2894,21 @@
         <v>170</v>
       </c>
       <c r="W19" t="n">
-        <v>39</v>
+        <v>41.92</v>
       </c>
       <c r="X19" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="Y19" t="n">
-        <v>6</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="Z19" t="inlineStr">
         <is>
-          <t>Engineers / Engineering employees</t>
+          <t>Employees in a manufacturing and engineering firm (nonmanagement team members)</t>
         </is>
       </c>
       <c r="AA19" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="AB19" t="n">
         <v>1</v>
@@ -2923,12 +2923,12 @@
       </c>
       <c r="AF19" t="inlineStr">
         <is>
-          <t>Marrone et al., 2007</t>
+          <t>Ancona and Caldwell’s (1992)</t>
         </is>
       </c>
       <c r="AG19" t="inlineStr">
         <is>
-          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
+          <t>We closely followed Ancona and Caldwell’s (1992) development of boundary-spanning items and selected 13 items from their research to assess the extent to which team members engaged in various boundary-spanning behaviors aimed at establishing and maintaining relationships with key external parties. Two of our constructs, supportive coaching and boundary-spanning self-efficacy, used traditional Likert scales (1 = strongly disagree to 5 = strongly agree), whereas our other two constructs utilized alternative anchor points (boundary spanning behavior, 1 = a very small extent to 5 = a very great extent; job satisfaction, 1 = very dissatisfied to 5 = very satisfied).</t>
         </is>
       </c>
       <c r="AH19" t="n">
@@ -2945,11 +2945,6 @@
           <t>1 = Self-report</t>
         </is>
       </c>
-      <c r="AL19" t="inlineStr">
-        <is>
-          <t>Subordinate rating of team leader/lead coaching behavior</t>
-        </is>
-      </c>
       <c r="AM19" t="inlineStr">
         <is>
           <t>Morgeson, 2005</t>
@@ -2957,7 +2952,7 @@
       </c>
       <c r="AN19" t="inlineStr">
         <is>
-          <t>Four-item scale developed for this study based on Morgeson (2005) asking employees to rate their lead's encouragement and empowerment of boundary spanning (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
+          <t>We relied on previous studies assessing supportive-coaching behaviors of encouragement and empowerment (e.g., Morgeson, 2005), as well as our discussions and interviews of organizational personnel, to develop a four-item scale for the purposes of this study that asked respondents to rate the extent to which they agreed that their lead encouraged and empowered employee engagement in boundary spanning. Two of our constructs, supportive coaching and boundary-spanning self-efficacy, used traditional Likert scales (1 = strongly disagree to 5 = strongly agree), whereas our other two constructs utilized alternative anchor points (boundary spanning behavior, 1 = a very small extent to 5 = a very great extent; job satisfaction, 1 = very dissatisfied to 5 = very satisfied).</t>
         </is>
       </c>
       <c r="AO19" t="inlineStr">
@@ -2966,13 +2961,13 @@
         </is>
       </c>
       <c r="AP19" t="n">
-        <v>3.48</v>
+        <v>2.62</v>
       </c>
       <c r="AQ19" t="n">
-        <v>0.65</v>
+        <v>0.83</v>
       </c>
       <c r="AR19" t="n">
-        <v>0.88</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AS19" t="inlineStr">
         <is>
@@ -3016,7 +3011,7 @@
       </c>
       <c r="Q20" t="inlineStr">
         <is>
-          <t>1 = Cross-sectional design</t>
+          <t>2 = Longitudinal design</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -3033,21 +3028,21 @@
         <v>170</v>
       </c>
       <c r="W20" t="n">
-        <v>39</v>
+        <v>41.92</v>
       </c>
       <c r="X20" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="Y20" t="n">
-        <v>6</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>Engineers / Engineering employees</t>
+          <t>Employees in a manufacturing and engineering firm (nonmanagement team members)</t>
         </is>
       </c>
       <c r="AA20" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="AB20" t="n">
         <v>1</v>
@@ -3062,12 +3057,12 @@
       </c>
       <c r="AF20" t="inlineStr">
         <is>
-          <t>Marrone et al., 2007</t>
+          <t>Ancona and Caldwell’s (1992)</t>
         </is>
       </c>
       <c r="AG20" t="inlineStr">
         <is>
-          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
+          <t>We closely followed Ancona and Caldwell’s (1992) development of boundary-spanning items and selected 13 items from their research to assess the extent to which team members engaged in various boundary-spanning behaviors aimed at establishing and maintaining relationships with key external parties. Two of our constructs, supportive coaching and boundary-spanning self-efficacy, used traditional Likert scales (1 = strongly disagree to 5 = strongly agree), whereas our other two constructs utilized alternative anchor points (boundary spanning behavior, 1 = a very small extent to 5 = a very great extent; job satisfaction, 1 = very dissatisfied to 5 = very satisfied).</t>
         </is>
       </c>
       <c r="AH20" t="n">
@@ -3091,7 +3086,7 @@
       </c>
       <c r="AN20" t="inlineStr">
         <is>
-          <t>Six-item scale from Marrone et al. (2007) assessing confidence in ability to effectively carry out and manage boundary-spanning behaviors (1 = strongly disagree to 5 = strongly agree; alpha = 0.95).</t>
+          <t>A previously established six-item scale from Marrone et al. (2007) was used to assess the extent to which team members agreed with statements regarding their confidence in their ability to effectively carry out and manage boundary-spanning behaviors. Two of our constructs, supportive coaching and boundary-spanning self-efficacy, used traditional Likert scales (1 = strongly disagree to 5 = strongly agree), whereas our other two constructs utilized alternative anchor points (boundary spanning behavior, 1 = a very small extent to 5 = a very great extent; job satisfaction, 1 = very dissatisfied to 5 = very satisfied).</t>
         </is>
       </c>
       <c r="AO20" t="inlineStr">
@@ -3100,13 +3095,13 @@
         </is>
       </c>
       <c r="AP20" t="n">
-        <v>3.48</v>
+        <v>2.62</v>
       </c>
       <c r="AQ20" t="n">
-        <v>0.65</v>
+        <v>0.83</v>
       </c>
       <c r="AR20" t="n">
-        <v>0.88</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AS20" t="inlineStr">
         <is>
@@ -3150,7 +3145,7 @@
       </c>
       <c r="Q21" t="inlineStr">
         <is>
-          <t>1 = Cross-sectional design</t>
+          <t>2 = Longitudinal design</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -3167,21 +3162,21 @@
         <v>170</v>
       </c>
       <c r="W21" t="n">
-        <v>39</v>
+        <v>41.92</v>
       </c>
       <c r="X21" t="n">
-        <v>21</v>
+        <v>10</v>
       </c>
       <c r="Y21" t="n">
-        <v>6</v>
+        <v>9.039999999999999</v>
       </c>
       <c r="Z21" t="inlineStr">
         <is>
-          <t>Engineers / Engineering employees</t>
+          <t>Employees in a manufacturing and engineering firm (nonmanagement team members)</t>
         </is>
       </c>
       <c r="AA21" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="AB21" t="n">
         <v>1</v>
@@ -3196,12 +3191,12 @@
       </c>
       <c r="AF21" t="inlineStr">
         <is>
-          <t>Marrone et al., 2007</t>
+          <t>Ancona and Caldwell’s (1992)</t>
         </is>
       </c>
       <c r="AG21" t="inlineStr">
         <is>
-          <t>Eight-item boundary-spanning behavior scale adapted from Marrone et al. (2007) and Ancona &amp; Caldwell (1992) capturing external communication and coordination across team boundaries (1 = strongly disagree to 5 = strongly agree; alpha = 0.88).</t>
+          <t>We closely followed Ancona and Caldwell’s (1992) development of boundary-spanning items and selected 13 items from their research to assess the extent to which team members engaged in various boundary-spanning behaviors aimed at establishing and maintaining relationships with key external parties. Two of our constructs, supportive coaching and boundary-spanning self-efficacy, used traditional Likert scales (1 = strongly disagree to 5 = strongly agree), whereas our other two constructs utilized alternative anchor points (boundary spanning behavior, 1 = a very small extent to 5 = a very great extent; job satisfaction, 1 = very dissatisfied to 5 = very satisfied).</t>
         </is>
       </c>
       <c r="AH21" t="n">
@@ -3220,12 +3215,12 @@
       </c>
       <c r="AM21" t="inlineStr">
         <is>
-          <t>Bacharach et al., 1991</t>
+          <t>Job Satisfaction Relative to Expectations instrument (Bacharach et al., 1991)</t>
         </is>
       </c>
       <c r="AN21" t="inlineStr">
         <is>
-          <t>Five-item Job Satisfaction Relative to Expectations instrument from Bacharach et al. (1991) rated on a 5-point scale (1 = very dissatisfied to 5 = very satisfied; alpha = 0.88).</t>
+          <t>Survey items for this measure were from the five-item Job Satisfaction Relative to Expectations instrument (Bacharach et al., 1991). The measure assesses the extent of agreement between broad satisfaction elements of a job relative to employee expectation. Two of our constructs, supportive coaching and boundary-spanning self-efficacy, used traditional Likert scales (1 = strongly disagree to 5 = strongly agree), whereas our other two constructs utilized alternative anchor points (boundary spanning behavior, 1 = a very small extent to 5 = a very great extent; job satisfaction, 1 = very dissatisfied to 5 = very satisfied).</t>
         </is>
       </c>
       <c r="AO21" t="inlineStr">
@@ -3234,13 +3229,13 @@
         </is>
       </c>
       <c r="AP21" t="n">
-        <v>3.48</v>
+        <v>2.62</v>
       </c>
       <c r="AQ21" t="n">
-        <v>0.65</v>
+        <v>0.83</v>
       </c>
       <c r="AR21" t="n">
-        <v>0.88</v>
+        <v>0.9399999999999999</v>
       </c>
       <c r="AS21" t="inlineStr">
         <is>
@@ -3335,7 +3330,7 @@
       </c>
       <c r="AE22" t="inlineStr">
         <is>
-          <t>Peer ratings across consulting teammates justified by median rwg = 0.80, ICC(1) = 0.28, ICC(2) = 0.71.</t>
+          <t>Peer ratings aggregated across consulting team members rating each individual teammate (median rwg = .80, ICC[1] = .28, ICC[2] = .71).</t>
         </is>
       </c>
       <c r="AF22" t="inlineStr">
@@ -3345,7 +3340,7 @@
       </c>
       <c r="AG22" t="inlineStr">
         <is>
-          <t>Six items adapted from Ancona and Caldwell (1992) capturing individual team member boundary-spanning behaviors across client, faculty advisor, and external organizational interfaces.</t>
+          <t>Closely following existing research, we measured individual boundary-spanning behavior with six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context. Team members rated the degree to which each of their teammates engaged in boundary-spanning behaviors (1, "not at all," to 5, "to a very great extent"). A principal components analysis yielded a single factor (alpha = .86).</t>
         </is>
       </c>
       <c r="AH22" t="n">
@@ -3369,7 +3364,7 @@
       </c>
       <c r="AN22" t="inlineStr">
         <is>
-          <t>Six items assessing the extent to which participants perceived boundary-spanning behaviors as an expected part of their role responsibilities (alpha = 0.86).</t>
+          <t>In accordance with role theory, we had all participants rate the extent to which they perceived each of the six boundary-spanning behaviors as an expected part of their responsibilities (1, "not at all," to 5, "to a very great extent"). Principal components analysis yielded a single factor (alpha = .86).</t>
         </is>
       </c>
       <c r="AO22" t="inlineStr">
@@ -3479,7 +3474,7 @@
       </c>
       <c r="AE23" t="inlineStr">
         <is>
-          <t>Peer ratings across consulting teammates justified by median rwg = 0.80, ICC(1) = 0.28, ICC(2) = 0.71.</t>
+          <t>Peer ratings aggregated across consulting team members rating each individual teammate (median rwg = .80, ICC[1] = .28, ICC[2] = .71).</t>
         </is>
       </c>
       <c r="AF23" t="inlineStr">
@@ -3489,7 +3484,7 @@
       </c>
       <c r="AG23" t="inlineStr">
         <is>
-          <t>Six items adapted from Ancona and Caldwell (1992) capturing individual team member boundary-spanning behaviors across client, faculty advisor, and external organizational interfaces.</t>
+          <t>Closely following existing research, we measured individual boundary-spanning behavior with six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context. Team members rated the degree to which each of their teammates engaged in boundary-spanning behaviors (1, "not at all," to 5, "to a very great extent"). A principal components analysis yielded a single factor (alpha = .86).</t>
         </is>
       </c>
       <c r="AH23" t="n">
@@ -3513,7 +3508,7 @@
       </c>
       <c r="AN23" t="inlineStr">
         <is>
-          <t>Eight-item scale adapted from Parker (1998) role breadth self-efficacy measuring confidence in engaging in boundary-spanning behaviors (alpha = 0.92).</t>
+          <t>We measured boundary-spanning self-efficacy by asking team members to rate their confidence in their ability to successfully engage in a variety of boundary-spanning behaviors. Scale items were based in part upon Parker's (1998) role breadth self-efficacy scale, which asks respondents to rate how confident they feel about contacting individuals outside of their own work units. Eight items were rated on a five-point disagree/agree Likert scale, and principal components analysis yielded a single factor (alpha = .92).</t>
         </is>
       </c>
       <c r="AO23" t="inlineStr">
@@ -3623,7 +3618,7 @@
       </c>
       <c r="AE24" t="inlineStr">
         <is>
-          <t>Peer ratings across consulting teammates justified by median rwg = 0.80, ICC(1) = 0.28, ICC(2) = 0.71.</t>
+          <t>Peer ratings aggregated across consulting team members rating each individual teammate (median rwg = .80, ICC[1] = .28, ICC[2] = .71).</t>
         </is>
       </c>
       <c r="AF24" t="inlineStr">
@@ -3633,7 +3628,7 @@
       </c>
       <c r="AG24" t="inlineStr">
         <is>
-          <t>Six items adapted from Ancona and Caldwell (1992) capturing individual team member boundary-spanning behaviors across client, faculty advisor, and external organizational interfaces.</t>
+          <t>Closely following existing research, we measured individual boundary-spanning behavior with six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context. Team members rated the degree to which each of their teammates engaged in boundary-spanning behaviors (1, "not at all," to 5, "to a very great extent"). A principal components analysis yielded a single factor (alpha = .86).</t>
         </is>
       </c>
       <c r="AH24" t="n">
@@ -3652,12 +3647,12 @@
       </c>
       <c r="AM24" t="inlineStr">
         <is>
-          <t>Williams &amp; O'Reilly (1998)</t>
+          <t>Williams &amp; O'Reilly, 1998</t>
         </is>
       </c>
       <c r="AN24" t="inlineStr">
         <is>
-          <t>Demographic control variable coded as Asian = 1 and other = 0.</t>
+          <t>Previous research has shown effects among demographic attributes and employee attitudes and behaviors (Williams &amp; O'Reilly, 1998). Consequently, we included Asian ethnicity (1, "Asian," and 0, "other"), and GMAT score (a continuous score) as controls when predicting individual boundary-spanning behavior.</t>
         </is>
       </c>
       <c r="AO24" t="inlineStr">
@@ -3767,7 +3762,7 @@
       </c>
       <c r="AE25" t="inlineStr">
         <is>
-          <t>Peer ratings across consulting teammates justified by median rwg = 0.80, ICC(1) = 0.28, ICC(2) = 0.71.</t>
+          <t>Peer ratings aggregated across consulting team members rating each individual teammate (median rwg = .80, ICC[1] = .28, ICC[2] = .71).</t>
         </is>
       </c>
       <c r="AF25" t="inlineStr">
@@ -3777,7 +3772,7 @@
       </c>
       <c r="AG25" t="inlineStr">
         <is>
-          <t>Six items adapted from Ancona and Caldwell (1992) capturing individual team member boundary-spanning behaviors across client, faculty advisor, and external organizational interfaces.</t>
+          <t>Closely following existing research, we measured individual boundary-spanning behavior with six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context. Team members rated the degree to which each of their teammates engaged in boundary-spanning behaviors (1, "not at all," to 5, "to a very great extent"). A principal components analysis yielded a single factor (alpha = .86).</t>
         </is>
       </c>
       <c r="AH25" t="n">
@@ -3794,11 +3789,6 @@
           <t>4 = Objective / Sociometric</t>
         </is>
       </c>
-      <c r="AL25" t="inlineStr">
-        <is>
-          <t>Continuous standardized test score</t>
-        </is>
-      </c>
       <c r="AM25" t="inlineStr">
         <is>
           <t>GMAT score</t>
@@ -3806,7 +3796,7 @@
       </c>
       <c r="AN25" t="inlineStr">
         <is>
-          <t>Continuous Graduate Management Admission Test (GMAT) cognitive ability score used as an individual control variable.</t>
+          <t>Consequently, we included Asian ethnicity (1, "Asian," and 0, "other"), and GMAT score (a continuous score) as controls when predicting individual boundary-spanning behavior.</t>
         </is>
       </c>
       <c r="AO25" t="inlineStr">
@@ -3916,7 +3906,7 @@
       </c>
       <c r="AE26" t="inlineStr">
         <is>
-          <t>Peer ratings across consulting teammates justified by median rwg = 0.80, ICC(1) = 0.28, ICC(2) = 0.71.</t>
+          <t>Peer ratings aggregated across consulting team members rating each individual teammate (median rwg = .80, ICC[1] = .28, ICC[2] = .71).</t>
         </is>
       </c>
       <c r="AF26" t="inlineStr">
@@ -3926,7 +3916,7 @@
       </c>
       <c r="AG26" t="inlineStr">
         <is>
-          <t>Six items adapted from Ancona and Caldwell (1992) capturing individual team member boundary-spanning behaviors across client, faculty advisor, and external organizational interfaces.</t>
+          <t>Closely following existing research, we measured individual boundary-spanning behavior with six items adapted directly from Ancona and Caldwell's (1992) study and modified to reflect the current consulting team context. Team members rated the degree to which each of their teammates engaged in boundary-spanning behaviors (1, "not at all," to 5, "to a very great extent"). A principal components analysis yielded a single factor (alpha = .86).</t>
         </is>
       </c>
       <c r="AH26" t="n">
@@ -3950,7 +3940,7 @@
       </c>
       <c r="AN26" t="inlineStr">
         <is>
-          <t>Three-item role overload scale adapted from Beehr et al. (1976) rated on a 5-point Likert scale (alpha = 0.83).</t>
+          <t>Three items were adapted from Beehr et al. (1976) and modified for the current context. They were rated on a five-point disagree/agree Likert scale. A principal components analysis yielded a single factor (alpha = .83).</t>
         </is>
       </c>
       <c r="AO26" t="inlineStr">
@@ -4011,7 +4001,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>The unit of statistical analysis is the business organization (N = 62 publicly held U.S. corporations on the Russell 1000 index). The 62 Public Affairs Managers served merely as single key informants evaluating the firm's macro-level relationships with public interest groups using firm-referent items (e.g., The firm avoids close contact with this socio-political actor), violating Screening Rule 4 and Rule 5 (Proxy Guardrail). Verbatim Evidence: [p. 58] "A survey of 62 Public Affairs Managers in publicly held U.S. corporations finds that organizations adopt relational styles similar to those theorized in studies of inter-organizational conflict, organizational communication and stakeholder management." [p. 62] "The organizations participating in this study were large, U.S. companies listed on the Russell 1000 index from a variety of industries... A limitation of the study is that only one manager responded for each organization. The vulnerability inherent in this practice is that the manager's understanding reflected in the survey may not be representative of the organization's practices."</t>
+          <t>The unit of statistical analysis is the business organization (N = 62 publicly held U.S. corporations on the Russell 1000 index), where 62 Public Affairs Managers served as single key informants rating firm-level relational tendencies using firm-referent items (Table 2, p. 14) and company multidimensional scaling coordinates (Table 6, p. 16; Table 9, p. 18). Verbatim Evidence: "[Abstract, p. 7] A survey of 62 Public Affairs Managers in publicly held U.S. corporations finds that organizations adopt relational styles similar to those theorized in studies of inter-organizational conflict, organizational communication and stakeholder management." "[Footnote 3, p. 13] The organizations participating in this study were large, U.S. companies listed on the Russell 1000 index from a variety of industries. Although the sample size is relatively small, it is well beyond the requirements for applying the central limit theorem and the respondents and non-respondents were not significantly different on any of several demographic variables, including size and financial performance measures. A limitation of the study is that only one manager responded for each organization. The vulnerability inherent in this practice is that the manager's understanding reflected in the survey may not be representative of the organization's practices." "[Table 2, p. 14] The firm avoids close contact with this socio-political actor. The firm's strategy for managing this socio-political actor is to maintain distance. The firm is not likely to conceal its intentions from this socio-political actor."</t>
         </is>
       </c>
     </row>
@@ -4036,7 +4026,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>The study surveys 193 county human service managers across five San Francisco Bay Area departments and measures managerial boundary spanning, but reports NO bivariate zero-order Pearson correlation matrix (r) involving boundary spanning. The only statistical results reported are multivariate ordinal logistic regressions with odds ratios (Table 4). Under Screening Rule 7, studies lacking extractable bivariate zero-order effect sizes must be excluded under Code 1. Verbatim Evidence: [p. 115] "A 2015 survey of 193 managers from five San Francisco Bay Area county human service departments examined the relationship between contract-based service coordination... and the predictors of managerial role, involvement, and boundary spanning. Multivariate regression results suggested that county managers identified fewer service coordination challenges if they were at the executive and program levels, had greater contract involvement, and engaged in contract-focused boundary spanning." [p. 122] "Bivariate Pearson, Spearman, and phi correlation tests did not indicate any problematic collinearity among independent variables (e.g., &gt; 0.33). Nor were the dependent variables highly correlated with any of the independent or control variables (i.e., all &gt; 0.21)."</t>
+          <t>The study surveys 193 county human service managers across five San Francisco Bay Area county departments and measures managerial boundary spanning (Table 3, p. 121: n = 180, Mean = 2.17, SD = 0.67), but reports NO bivariate zero-order correlations (r) or convertible t/chi-square statistics involving boundary spanning. The only statistical models linking boundary spanning to other variables are multivariate ordinal logistic regressions reporting adjusted odds ratios (Table 4, p. 122). Verbatim Evidence: "[Abstract, p. 115] A 2015 survey of 193 managers from five San Francisco Bay Area county human service departments examined the relationship between contract-based service coordination (i.e., structuring cross-sector services, coordinating client referrals and eligibility, overseeing EBP implementation) and the predictors of managerial role, involvement, and boundary spanning. Multivariate regression results suggested that county managers identified fewer service coordination challenges if they were at the executive and program levels, had greater contract involvement, and engaged in contract-focused boundary spanning." "[Analyses, p. 121] Three ordinal logistic regressions, with standard errors clustered by county organization, were conducted to examine associations between managerial factors and each of the dependent variables." "[Analyses, p. 121] Bivariate Pearson, Spearman, and phi correlation tests did not indicate any problematic collinearity among independent variables (e.g., &gt; 0.33). Nor were the dependent variables highly correlated with any of the independent or control variables (i.e., all &gt; 0.21)."</t>
         </is>
       </c>
     </row>

</xml_diff>